<commit_message>
Update October 2026 policy evidence, city contribution bases and guides
</commit_message>
<xml_diff>
--- a/public/downloads/import-templates/employment-cost.xlsx
+++ b/public/downloads/import-templates/employment-cost.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批量填写" sheetId="1" r:id="R20d927bf6543479f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="批量填写" sheetId="1" r:id="R9eeba30d3c774d08"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,18 +21,18 @@
     <x:font>
       <x:sz val="11"/>
       <x:color rgb="FF273444"/>
-      <x:name val="Microsoft YaHei"/>
+      <x:name val="Noto Sans CJK SC"/>
     </x:font>
     <x:font>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Microsoft YaHei"/>
+      <x:name val="Noto Sans CJK SC"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Microsoft YaHei"/>
+      <x:name val="Noto Sans CJK SC"/>
     </x:font>
   </x:fonts>
   <x:fills count="4">
@@ -54,7 +54,13 @@
     </x:fill>
   </x:fills>
   <x:borders count="1">
-    <x:border/>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>

</xml_diff>